<commit_message>
Add 30 commercial listicle keywords across 15 industries
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -573,6 +573,726 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for schools</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>best keynote speaker for school leaders</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for schools</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for churches</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for nonprofits</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>best keynote speaker for church leaders</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for aged care</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for aged care</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for hospitals</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for healthcare</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for construction companies</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for construction</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for mining companies</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for mining</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for agriculture</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for agribusiness</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for manufacturing</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for manufacturing</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for accounting firms</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for accounting firms</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for law firms</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for law firms</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for engineering firms</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for architecture firms</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for hospitality</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for hotels</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for retail</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>top leadership consultants for retail</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for real estate</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>best leadership speaker for local government</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update blog queue: working genius tips for leaders -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -514,11 +514,15 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: working genius tips for leaders -> SKIP
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -527,7 +527,11 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Skipped per user request 2026-03-24</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: skip best leadership facilitator Brisbane + difficult conversations training Australia
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
@@ -555,7 +555,11 @@
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Skipped per user request 2026-03-24</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -570,7 +574,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -579,7 +583,11 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Skipped per user request 2026-03-24</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for schools -> SKIP
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
@@ -611,7 +611,11 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Skipped per user request 2026-03-24</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: best keynote speaker for school leaders -> SKIP
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -630,7 +630,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
@@ -639,7 +639,11 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Skipped per user request 2026-03-24</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for schools -> SKIP
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -658,7 +658,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
@@ -667,7 +667,11 @@
       <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Skipped per user request 2026-03-24</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for churches -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -686,11 +686,15 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add 145 new keywords to blog queue (thought leaders, keynote speakers, industry leadership)
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1325,6 +1325,2471 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on operations</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on boredom</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in independent private schools</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on supply chain</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on second-in-command leadership</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in credit unions</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on logistics</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on leadership transitions</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in aged care facilities</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on manufacturing</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on founder succession</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in mutual banks</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on quality assurance</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on reverse mentoring</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in home care</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on HR</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on overcommunication</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in building societies</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on people and culture</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on leadership under scrutiny</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in disability service providers</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on learning and development</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on unwritten rules</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in Catholic systemic schools</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on workplace health and safety</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on decision avoidance</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in Catholic independent schools</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on finance</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on apprenticeship</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in mid-tier accounting firms</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on accounting</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on execution timing</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in pathology labs</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on payroll</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on performance reviews</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in residential property management</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on procurement</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on inherited teams</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in boutique accounting firms</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on risk management</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on ego and humility</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in regional law firms</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on sales</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on consensus</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in radiology and imaging groups</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on business development</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on role switching</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in commercial property management</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on partnerships</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on organisational overcorrection</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in facilities management companies</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on marketing</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on invisible workload</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in fertility clinics</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on brand strategy</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on outgrowing your role</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in FinTech companies</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on digital marketing</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on loyalty</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in pharmaceutical manufacturing</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on public relations</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on low-urgency leadership</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in renewable energy companies</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on corporate communications</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on middle management</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in boutique hotel groups</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on events management</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on parenting and leadership</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in mid-sized commercial builders</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on legal</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on leading without data</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in medical device manufacturers</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on compliance</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on best practice</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in civil construction firms</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on governance</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on institutional courage</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in solar installation companies</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on IT</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on work-life integration</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in resort properties</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on software engineering</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on understimulation</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in HealthTech companies</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on data and analytics</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on leader formation</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in cosmetics and personal care manufacturing</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on cybersecurity</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on productive disagreement</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in electrical contracting companies</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on product management</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on competing values</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in wind farm operators</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on strategy</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on mediocrity</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in RSL and services clubs</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on project management</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on leading creatives</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in EdTech companies</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on change management</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on credibility</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in food and beverage manufacturing</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on customer service</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on organisational memory</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in freight and trucking companies</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on customer success</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on small team leadership</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in automotive dealer groups</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on facilities management</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on return to work</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in large farming operations</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on investor relations</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on turnaround leadership</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in regional pharmacy chains</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on government relations</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on empathy and avoidance</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in warehousing and 3PL providers</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on sustainability</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on leadership language</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in feedlot operations</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on community engagement</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on ethical grey zones</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in hardware and building supply chains</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on R&amp;D</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on introverted leadership</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in regional bus companies</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on design and creative</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on alumni and leavers</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in abattoirs and meat processing</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on fundraising</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on meeting-free culture</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in furniture retailer groups</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Best thought leaders globally on pastoral care and wellbeing</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on code-switching</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in Anglican and Episcopal diocese offices</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on system failure vs individual failure</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in housing associations</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on internal rebranding</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in Catholic diocese offices</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on patience</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in homelessness services</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on organisational comparison</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in Pentecostal network offices</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Best keynote speakers globally on legacy</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Best thought leaders on leadership in youth services</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for nonprofits -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -714,11 +714,15 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for nonprofits -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -714,20 +714,42 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-nonprofits-20260324</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>3380</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>17 consultants listed. Full content published to Wix. 37 LinkedIn tags.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: best keynote speaker for church leaders -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -764,16 +764,42 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-keynote-speakers-for-church-leaders-2026</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>5875</v>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>50 speakers listed. Full content published to Wix. 45 LinkedIn tags. Buffer: X, FB, IG, Threads, GBP, Bluesky scheduled. Pinterest skipped (no boards).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for aged care -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -814,11 +814,15 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for aged care -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -814,19 +814,37 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-aged-care-20260324</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>5587</v>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for aged care -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -860,11 +860,15 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for aged care -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -860,19 +860,37 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-aged-care-20260324</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>5088</v>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for hospitals -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -906,11 +906,15 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for hospitals -> WRITTEN
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -906,19 +906,33 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-hospitals-20260324</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>6030</v>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for hospitals -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -906,7 +906,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -924,7 +924,11 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-hospitals-20260324</t>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for healthcare -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -952,11 +952,15 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for healthcare -> PUBLISHED + LinkedIn post
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -952,20 +952,42 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-healthcare-20260325</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>5011</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Published to Wix, Buffer scheduled (X, FB, IG, Threads, GBP, Bluesky). Pinterest skipped (no boards). LinkedIn manual.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Queue: healthcare consultants -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -977,15 +977,15 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-healthcare-20260325</t>
+          <t>https://www.consultclarity.org/post/50-top-leadership-consultants-for-healthcare-2026-1</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>5011</v>
+        <v>5786</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Published to Wix, Buffer scheduled (X, FB, IG, Threads, GBP, Bluesky). Pinterest skipped (no boards). LinkedIn manual.</t>
+          <t>50 consultants. Full Wix. 41 LinkedIn tags. Buffer scheduled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for construction companies -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1002,11 +1002,15 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for construction companies -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1002,20 +1002,42 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-construction-20260325</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>5940</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Published to Wix. 50 speakers, 773 Ricos nodes. LinkedIn post ready.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for construction -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1052,11 +1052,15 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for construction -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1052,19 +1052,33 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-construction-20260325</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>6654</v>
+      </c>
       <c r="J16" s="2" t="inlineStr"/>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for construction -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1070,7 +1070,11 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-construction-20260325</t>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for mining companies -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1098,11 +1098,15 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for mining companies -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1098,20 +1098,42 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-mining-companies-20260325</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>5574</v>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>50 entries. Published to Wix. Buffer scheduled 7/8 (TikTok daily limit).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for mining -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1148,11 +1148,15 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for mining -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1148,20 +1148,38 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-mining-20260325</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>5406</v>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>50 consultants listed. Images and carousel created.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for mining -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1166,7 +1166,11 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-mining-20260325</t>
@@ -1177,7 +1181,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>50 consultants listed. Images and carousel created.</t>
+          <t>50 consultants listed. Full content published to Wix (495 nodes). 45 LinkedIn tags. Buffer: X, FB, IG, Threads, GBP, Bluesky, YouTube scheduled. TikTok daily limit. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for agriculture -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1198,11 +1198,15 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for agriculture -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1198,19 +1198,33 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-agriculture-20260325</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>5339</v>
+      </c>
       <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for agriculture -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1216,7 +1216,11 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-agriculture-20260325</t>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for agribusiness -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1244,11 +1244,15 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for agribusiness -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1244,19 +1244,33 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-agribusiness-20260325</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>5024</v>
+      </c>
       <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Update blog queue: top leadership consultants for agribusiness -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1244,7 +1244,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1262,7 +1262,11 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
           <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-top-leadership-consultants-agribusiness-20260325</t>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for manufacturing -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1290,11 +1290,15 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Update blog queue: best leadership speaker for manufacturing -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1290,19 +1290,37 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-leadership-speakers-manufacturing-20260325</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>5068</v>
+      </c>
       <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Rebuild queue: 170 unique global industry thought leader keywords
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J179"/>
+  <dimension ref="A1:J194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1324,321 +1324,230 @@
       <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>top leadership consultants for manufacturing</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Best thought leaders in accounting</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for accounting firms</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Best thought leaders in hospitality</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>top leadership consultants for accounting firms</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Best thought leaders in law</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for law firms</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Best thought leaders in engineering</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>top leadership consultants for law firms</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Best thought leaders in architecture</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for engineering firms</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Best thought leaders in retail</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for architecture firms</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Best thought leaders in real estate</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for hospitality</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Best thought leaders in manufacturing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>top leadership consultants for hotels</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Best thought leaders in agriculture</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for retail</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mining</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>top leadership consultants for retail</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Best thought leaders in construction</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for real estate</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Best thought leaders in healthcare</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>best leadership speaker for local government</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Best thought leaders in aged care</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on operations</t>
+          <t>Best thought leaders in banking</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1655,7 +1564,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on boredom</t>
+          <t>Best thought leaders in insurance</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1672,7 +1581,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in independent private schools</t>
+          <t>Best thought leaders in consulting</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1689,7 +1598,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on supply chain</t>
+          <t>Best thought leaders in technology</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1706,7 +1615,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on second-in-command leadership</t>
+          <t>Best thought leaders in cybersecurity</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1723,7 +1632,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in credit unions</t>
+          <t>Best thought leaders in artificial intelligence</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1740,7 +1649,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on logistics</t>
+          <t>Best thought leaders in data and analytics</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1757,7 +1666,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on leadership transitions</t>
+          <t>Best thought leaders in software engineering</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1774,7 +1683,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in aged care facilities</t>
+          <t>Best thought leaders in product management</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1791,7 +1700,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on manufacturing</t>
+          <t>Best thought leaders in supply chain</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1808,7 +1717,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on founder succession</t>
+          <t>Best thought leaders in logistics</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1825,7 +1734,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in mutual banks</t>
+          <t>Best thought leaders in procurement</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1842,7 +1751,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on quality assurance</t>
+          <t>Best thought leaders in human resources</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1859,7 +1768,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on reverse mentoring</t>
+          <t>Best thought leaders in people and culture</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1876,7 +1785,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in home care</t>
+          <t>Best thought leaders in learning and development</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1893,7 +1802,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on HR</t>
+          <t>Best thought leaders in finance</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1910,7 +1819,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on overcommunication</t>
+          <t>Best thought leaders in investment management</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1927,7 +1836,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in building societies</t>
+          <t>Best thought leaders in venture capital</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1944,7 +1853,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on people and culture</t>
+          <t>Best thought leaders in private equity</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1961,7 +1870,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on leadership under scrutiny</t>
+          <t>Best thought leaders in mergers and acquisitions</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1978,7 +1887,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in disability service providers</t>
+          <t>Best thought leaders in risk management</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1995,7 +1904,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on learning and development</t>
+          <t>Best thought leaders in compliance</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2012,7 +1921,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on unwritten rules</t>
+          <t>Best thought leaders in governance</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2029,7 +1938,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in Catholic systemic schools</t>
+          <t>Best thought leaders in sustainability</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2046,7 +1955,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on workplace health and safety</t>
+          <t>Best thought leaders in ESG</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2063,7 +1972,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on decision avoidance</t>
+          <t>Best thought leaders in renewable energy</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2080,7 +1989,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in Catholic independent schools</t>
+          <t>Best thought leaders in oil and gas</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2097,7 +2006,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on finance</t>
+          <t>Best thought leaders in aviation</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2114,7 +2023,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on apprenticeship</t>
+          <t>Best thought leaders in shipping and maritime</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2131,7 +2040,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in mid-tier accounting firms</t>
+          <t>Best thought leaders in telecommunications</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2148,7 +2057,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on accounting</t>
+          <t>Best thought leaders in media and entertainment</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2165,7 +2074,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on execution timing</t>
+          <t>Best thought leaders in advertising</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2182,7 +2091,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in pathology labs</t>
+          <t>Best thought leaders in public relations</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2199,7 +2108,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on payroll</t>
+          <t>Best thought leaders in marketing</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2216,7 +2125,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on performance reviews</t>
+          <t>Best thought leaders in digital marketing</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2233,7 +2142,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in residential property management</t>
+          <t>Best thought leaders in sales</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2250,7 +2159,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on procurement</t>
+          <t>Best thought leaders in customer experience</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2267,7 +2176,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on inherited teams</t>
+          <t>Best thought leaders in customer success</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2284,7 +2193,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in boutique accounting firms</t>
+          <t>Best thought leaders in project management</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2301,7 +2210,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on risk management</t>
+          <t>Best thought leaders in change management</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2318,7 +2227,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on ego and humility</t>
+          <t>Best thought leaders in strategy</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2335,7 +2244,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in regional law firms</t>
+          <t>Best thought leaders in innovation</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2352,7 +2261,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on sales</t>
+          <t>Best thought leaders in design and creative</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2369,7 +2278,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on consensus</t>
+          <t>Best thought leaders in education</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2386,7 +2295,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in radiology and imaging groups</t>
+          <t>Best thought leaders in higher education</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2403,7 +2312,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on business development</t>
+          <t>Best thought leaders in independent schools</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2420,7 +2329,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on role switching</t>
+          <t>Best thought leaders in early childhood education</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2437,7 +2346,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in commercial property management</t>
+          <t>Best thought leaders in nonprofits</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2454,7 +2363,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on partnerships</t>
+          <t>Best thought leaders in social enterprise</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2471,7 +2380,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on organisational overcorrection</t>
+          <t>Best thought leaders in government</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2488,7 +2397,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in facilities management companies</t>
+          <t>Best thought leaders in local government</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2505,7 +2414,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on marketing</t>
+          <t>Best thought leaders in defence</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2522,7 +2431,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on invisible workload</t>
+          <t>Best thought leaders in policing and law enforcement</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2539,7 +2448,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in fertility clinics</t>
+          <t>Best thought leaders in emergency services</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2556,7 +2465,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on brand strategy</t>
+          <t>Best thought leaders in pharmaceuticals</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2573,7 +2482,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on outgrowing your role</t>
+          <t>Best thought leaders in biotech</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2590,7 +2499,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in FinTech companies</t>
+          <t>Best thought leaders in medical devices</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2607,7 +2516,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on digital marketing</t>
+          <t>Best thought leaders in veterinary</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2624,7 +2533,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on loyalty</t>
+          <t>Best thought leaders in dental</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2641,7 +2550,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in pharmaceutical manufacturing</t>
+          <t>Best thought leaders in mental health</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2658,7 +2567,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on public relations</t>
+          <t>Best thought leaders in disability services</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2675,7 +2584,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on low-urgency leadership</t>
+          <t>Best thought leaders in childcare</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2692,7 +2601,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in renewable energy companies</t>
+          <t>Best thought leaders in housing</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2709,7 +2618,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on corporate communications</t>
+          <t>Best thought leaders in sports</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2726,7 +2635,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on middle management</t>
+          <t>Best thought leaders in fitness and wellness</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2743,7 +2652,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in boutique hotel groups</t>
+          <t>Best thought leaders in food and beverage</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2760,7 +2669,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on events management</t>
+          <t>Best thought leaders in franchising</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2777,7 +2686,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on parenting and leadership</t>
+          <t>Best thought leaders in automotive</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2794,7 +2703,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in mid-sized commercial builders</t>
+          <t>Best thought leaders in transport</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2811,7 +2720,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on legal</t>
+          <t>Best thought leaders in railways</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2828,7 +2737,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on leading without data</t>
+          <t>Best thought leaders in property management</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2845,7 +2754,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in medical device manufacturers</t>
+          <t>Best thought leaders in facilities management</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2862,7 +2771,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on compliance</t>
+          <t>Best thought leaders in cleaning and maintenance</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2879,7 +2788,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on best practice</t>
+          <t>Best thought leaders in waste management</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2896,7 +2805,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in civil construction firms</t>
+          <t>Best thought leaders in water and utilities</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2913,7 +2822,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on governance</t>
+          <t>Best thought leaders in forestry</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2930,7 +2839,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on institutional courage</t>
+          <t>Best thought leaders in fisheries and aquaculture</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2947,7 +2856,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in solar installation companies</t>
+          <t>Best thought leaders in wine and spirits</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2964,7 +2873,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on IT</t>
+          <t>Best thought leaders in tourism</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2981,7 +2890,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on work-life integration</t>
+          <t>Best thought leaders in events management</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2998,7 +2907,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in resort properties</t>
+          <t>Best thought leaders in recruitment and staffing</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3015,7 +2924,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on software engineering</t>
+          <t>Best thought leaders in workplace health and safety</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3032,7 +2941,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on understimulation</t>
+          <t>Best thought leaders in industrial relations</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3049,7 +2958,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in HealthTech companies</t>
+          <t>Best thought leaders in organisational psychology</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3066,7 +2975,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on data and analytics</t>
+          <t>Best thought leaders in executive coaching</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3083,7 +2992,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on leader formation</t>
+          <t>Best thought leaders in board governance</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3100,7 +3009,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in cosmetics and personal care manufacturing</t>
+          <t>Best thought leaders in family business</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3117,7 +3026,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on cybersecurity</t>
+          <t>Best thought leaders in small business</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3134,7 +3043,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on productive disagreement</t>
+          <t>Best thought leaders in startups</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3151,7 +3060,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in electrical contracting companies</t>
+          <t>Best thought leaders in e-commerce</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3168,7 +3077,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on product management</t>
+          <t>Best thought leaders in SaaS</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3185,7 +3094,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on competing values</t>
+          <t>Best thought leaders in fintech</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3202,7 +3111,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in wind farm operators</t>
+          <t>Best thought leaders in edtech</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3219,7 +3128,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on strategy</t>
+          <t>Best thought leaders in healthtech</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3236,7 +3145,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on mediocrity</t>
+          <t>Best thought leaders in proptech</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3253,7 +3162,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in RSL and services clubs</t>
+          <t>Best thought leaders in agritech</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3270,7 +3179,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on project management</t>
+          <t>Best thought leaders in legaltech</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3287,7 +3196,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on leading creatives</t>
+          <t>Best thought leaders in regtech</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3304,7 +3213,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in EdTech companies</t>
+          <t>Best thought leaders in crypto and blockchain</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3321,7 +3230,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on change management</t>
+          <t>Best thought leaders in gaming</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3338,7 +3247,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on credibility</t>
+          <t>Best thought leaders in fashion</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3355,7 +3264,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in food and beverage manufacturing</t>
+          <t>Best thought leaders in luxury brands</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3372,7 +3281,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on customer service</t>
+          <t>Best thought leaders in beauty and cosmetics</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3389,7 +3298,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on organisational memory</t>
+          <t>Best thought leaders in publishing</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3406,7 +3315,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in freight and trucking companies</t>
+          <t>Best thought leaders in journalism</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3423,7 +3332,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on customer success</t>
+          <t>Best thought leaders in podcasting</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3440,7 +3349,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on small team leadership</t>
+          <t>Best thought leaders in film and television</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3457,7 +3366,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in automotive dealer groups</t>
+          <t>Best thought leaders in music</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3474,7 +3383,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on facilities management</t>
+          <t>Best thought leaders in performing arts</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3491,7 +3400,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on return to work</t>
+          <t>Best thought leaders in visual arts</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3508,7 +3417,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in large farming operations</t>
+          <t>Best thought leaders in museums and galleries</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3525,7 +3434,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on investor relations</t>
+          <t>Best thought leaders in libraries</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3542,7 +3451,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on turnaround leadership</t>
+          <t>Best thought leaders in faith-based organisations</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -3559,7 +3468,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in regional pharmacy chains</t>
+          <t>Best thought leaders in community development</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -3576,7 +3485,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on government relations</t>
+          <t>Best thought leaders in Indigenous leadership</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -3593,7 +3502,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on empathy and avoidance</t>
+          <t>Best thought leaders in women in leadership</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -3610,7 +3519,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in warehousing and 3PL providers</t>
+          <t>Best thought leaders in diversity and inclusion</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -3627,7 +3536,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on sustainability</t>
+          <t>Best thought leaders in remote and hybrid work</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -3644,7 +3553,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on leadership language</t>
+          <t>Best thought leaders in employee engagement</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -3661,7 +3570,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in feedlot operations</t>
+          <t>Best thought leaders in talent management</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -3678,7 +3587,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on community engagement</t>
+          <t>Best thought leaders in succession planning</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -3695,7 +3604,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on ethical grey zones</t>
+          <t>Best thought leaders in corporate culture</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -3712,7 +3621,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in hardware and building supply chains</t>
+          <t>Best thought leaders in teams and collaboration</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -3729,7 +3638,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on R&amp;D</t>
+          <t>Best thought leaders in conflict resolution</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -3746,7 +3655,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on introverted leadership</t>
+          <t>Best thought leaders in negotiation</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -3763,7 +3672,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in regional bus companies</t>
+          <t>Best thought leaders in emotional intelligence</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -3780,7 +3689,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on design and creative</t>
+          <t>Best thought leaders in resilience</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -3797,7 +3706,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on alumni and leavers</t>
+          <t>Best thought leaders in mindfulness and wellbeing</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -3814,7 +3723,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in abattoirs and meat processing</t>
+          <t>Best thought leaders in communications</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -3831,7 +3740,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on fundraising</t>
+          <t>Best thought leaders in public speaking</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -3848,7 +3757,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on meeting-free culture</t>
+          <t>Best thought leaders in storytelling</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -3865,7 +3774,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in furniture retailer groups</t>
+          <t>Best thought leaders in personal branding</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -3882,7 +3791,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Best thought leaders globally on pastoral care and wellbeing</t>
+          <t>Best thought leaders in career development</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -3899,7 +3808,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on code-switching</t>
+          <t>Best thought leaders in mentoring</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -3916,7 +3825,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in Anglican and Episcopal diocese offices</t>
+          <t>Best thought leaders in intergenerational leadership</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -3933,7 +3842,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on system failure vs individual failure</t>
+          <t>Best thought leaders in ethics and integrity</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -3950,7 +3859,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in housing associations</t>
+          <t>Best thought leaders in crisis management</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -3967,7 +3876,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on internal rebranding</t>
+          <t>Best thought leaders in turnaround leadership</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -3984,7 +3893,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in Catholic diocese offices</t>
+          <t>Best thought leaders in merging organisations</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4001,7 +3910,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on patience</t>
+          <t>Best thought leaders in scaling organisations</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4018,7 +3927,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in homelessness services</t>
+          <t>Best thought leaders in lean and continuous improvement</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4035,7 +3944,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on organisational comparison</t>
+          <t>Best thought leaders in quality management</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4052,7 +3961,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in Pentecostal network offices</t>
+          <t>Best thought leaders in operations</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4069,7 +3978,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Best keynote speakers globally on legacy</t>
+          <t>Best thought leaders in R&amp;D</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4086,7 +3995,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Best thought leaders on leadership in youth services</t>
+          <t>Best thought leaders in intellectual property</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4095,6 +4004,261 @@
         </is>
       </c>
       <c r="C179" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Best thought leaders in international business</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Best thought leaders in cross-cultural leadership</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Best thought leaders in social media</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Best thought leaders in influencer marketing</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Best thought leaders in content strategy</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Best thought leaders in brand strategy</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Best thought leaders in pricing strategy</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Best thought leaders in behavioural science</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Best thought leaders in neuroscience and leadership</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Best thought leaders in systems thinking</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Best thought leaders in complexity and adaptive leadership</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Best thought leaders in servant leadership</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Best thought leaders in values-based leadership</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Best thought leaders in purpose-driven leadership</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Best thought leaders in regenerative leadership</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in accounting -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1336,7 +1336,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: accounting -> SKIP, hospitality -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1336,12 +1336,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Already published: thought-leaders-accounting-usa</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1363,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: hospitality -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1363,12 +1363,40 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/50-best-thought-leaders-in-hospitality-2026</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>5815</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>50 entries, full pipeline complete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in law -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1413,7 +1413,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Skip law (exists), pick engineering -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1413,12 +1413,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Already published: thought-leaders-law-firm-leadership</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1440,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in engineering -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1440,12 +1440,40 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-engineering-20260325</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>5835</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>50 entries. Full content published to Wix (465 nodes). 48 LinkedIn tags. Buffer: X, FB, IG, Threads, GBP, Bluesky, TikTok, YouTube scheduled. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in architecture -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1490,7 +1490,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: thought leaders in architecture -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1490,13 +1490,31 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-architecture-20260326</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>6212</v>
       </c>
     </row>
     <row r="27">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in retail -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1530,7 +1530,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in retail -> WRITTEN
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1530,13 +1530,31 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-retail-20260326</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>6255</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in retail -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1530,7 +1530,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1544,6 +1544,11 @@
         </is>
       </c>
       <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
@@ -1555,6 +1560,11 @@
       </c>
       <c r="I27" t="n">
         <v>6255</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>50 entries. Full content published to Wix (498 nodes). 47 LinkedIn tags. Buffer: X, FB, IG, Threads, GBP, Bluesky, YouTube scheduled. TikTok daily limit. Pinterest skipped (no boards).</t>
+        </is>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in real estate -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1580,7 +1580,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: thought leaders in real estate -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1580,13 +1580,31 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-real-estate-20260326</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>7407</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Update blog queue: thought leaders in real estate -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1580,7 +1580,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1594,6 +1594,11 @@
         </is>
       </c>
       <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in manufacturing -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1625,7 +1625,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in manufacturing -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1625,12 +1625,40 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-manufacturing-20260326</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>5180</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>50 entries. Full content published to Wix (390 nodes). 48 LinkedIn tags. Buffer: X, FB, IG, Threads, GBP, Bluesky, TikTok, YouTube scheduled. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in agriculture -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1675,7 +1675,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in agriculture -> WRITTEN
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1675,13 +1675,31 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-agriculture-20260326</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>7324</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Update agriculture thought leaders status to PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1670,7 +1670,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>COMMERCIAL</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1689,6 +1689,11 @@
         </is>
       </c>
       <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in mining -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
@@ -699,7 +699,11 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Already published: 50 Best Keynote Speakers for Church Leaders (2026)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1720,7 +1724,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in mining -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1724,13 +1724,36 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-thought-leaders-mining-20260326</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>5221</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in construction -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1769,7 +1769,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in healthcare -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1791,7 +1791,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in healthcare -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1791,13 +1791,31 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-in-healthcare-20260326</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>6602</v>
       </c>
     </row>
     <row r="34">

</xml_diff>

<commit_message>
Update 'Best thought leaders in healthcare' status to PUBLISHED (2026-03-26)
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1791,7 +1791,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1805,6 +1805,11 @@
         </is>
       </c>
       <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in aged care -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1836,7 +1836,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: skipped aged care & banking, insurance -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1836,12 +1836,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Already published: 35 Best Thought Leaders in Residential Aged Care (2026)</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1863,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>SKIP</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Already published: 50 Essential Banking Thought Leaders on LinkedIn</t>
         </is>
       </c>
     </row>
@@ -1875,7 +1885,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: insurance -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1885,13 +1885,31 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-in-insurance-20260326</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>5520</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
Update blog queue: insurance -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1899,6 +1899,11 @@
         </is>
       </c>
       <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in consulting -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1930,7 +1930,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in technology -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1952,7 +1952,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 'Best thought leaders in technology' to PUBLISHED (2026-03-26)
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1952,10 +1952,15 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>2026-03-26</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in cybersecurity -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -1979,7 +1979,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in artificial intelligence -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2001,7 +2001,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in artificial intelligence -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2001,13 +2001,31 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-in-artificial-intelligence-20260327</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>6947</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in artificial intelligence -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>PUBLISHED</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2015,6 +2015,11 @@
         </is>
       </c>
       <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in data and analytics -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2046,7 +2046,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: best thought leaders in data and analytics -> WRITTEN + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2046,13 +2046,31 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-data-analytics-20260327</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>6796</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in software engineering -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2086,7 +2086,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: software engineering -> PUBLISHED + handoff + LinkedIn post
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2086,12 +2086,40 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-software-engineering-20260327</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>5916</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>50 entries. Full content published to Wix (625 nodes). 49 LinkedIn tags. Buffer: X, FB, IG, Threads, GBP, Bluesky, YouTube scheduled. TikTok daily limit. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in product management -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2136,7 +2136,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in product management -> PUBLISHED
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2136,12 +2136,40 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-product-management-20260327</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>6647</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Published to Wix. 50 items. LinkedIn post ready. Buffer posts scheduled.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 160 new keywords to blog queue
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J194"/>
+  <dimension ref="A1:J354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4740,6 +4740,2726 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Best thought leaders in enterprise saas</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Best thought leaders in ai and machine learning</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Best thought leaders in cloud infrastructure</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Best thought leaders in series b+ startups</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Best thought leaders in scaling platforms</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Best thought leaders in devops and platform engineering</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Best thought leaders in financial services</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Best thought leaders in investment banking</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Best thought leaders in wealth management</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Best thought leaders in asset management</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Best thought leaders in hedge funds</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Best thought leaders in private equity firms</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Best thought leaders in venture capital firms</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Best thought leaders in retail banking</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Best thought leaders in commercial banking</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Best thought leaders in superannuation and pension funds</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Best thought leaders in professional services</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Best thought leaders in big 4 accounting and consulting</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mid-tier accounting firms</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Best thought leaders in management consulting</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Best thought leaders in engineering consulting</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Best thought leaders in architecture firms</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Best thought leaders in recruitment and staffing agencies</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Best thought leaders in it consulting</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Best thought leaders in legal</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Best thought leaders in top-tier law firms</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mid-tier law firms</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Best thought leaders in boutique specialist law firms</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Best thought leaders in barristers chambers</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Best thought leaders in patent and ip law firms</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Best thought leaders in hospital networks and health systems</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Best thought leaders in aged care and senior living</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Best thought leaders in health insurance</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Best thought leaders in medical device companies</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mental health and allied health groups</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Best thought leaders in primary care networks</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Best thought leaders in private equity portfolio companies</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Best thought leaders in post-acquisition integration</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Best thought leaders in growth-stage portfolio companies</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Best thought leaders in turnaround and restructuring portfolio companies</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Best thought leaders in add-on acquisition integration</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Best thought leaders in pharmaceutical and biotech</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Best thought leaders in large pharma</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Best thought leaders in biotech startups</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Best thought leaders in clinical research organizations</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Best thought leaders in medical research institutes</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mining and resources</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Best thought leaders in iron ore and coal</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Best thought leaders in gold and precious metals</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Best thought leaders in lithium and critical minerals</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Best thought leaders in lng</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mining services contractors</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Best thought leaders in energy</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Best thought leaders in renewables</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Best thought leaders in utilities</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Best thought leaders in energy retail</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Best thought leaders in power generation</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Best thought leaders in real estate and property</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Best thought leaders in commercial property developers</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Best thought leaders in reits</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Best thought leaders in property management groups</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Best thought leaders in residential developers</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Best thought leaders in independent and private schools</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Best thought leaders in school associations and networks</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Best thought leaders in universities</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Best thought leaders in international schools</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Best thought leaders in catholic and faith-based school systems</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Best thought leaders in large nonprofits and faith-based organizations</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Best thought leaders in mega-churches</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Best thought leaders in international ngos</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Best thought leaders in large domestic charities</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Best thought leaders in denominational bodies</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Best thought leaders in community health organizations</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Best thought leaders in family offices</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Best thought leaders in single-family offices</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Best thought leaders in multi-family offices</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Best thought leaders in intergenerational wealth transfer families</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Best thought leaders in government and public sector</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Best thought leaders in federal government departments</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Best thought leaders in state government agencies</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Best thought leaders in major carriers</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Best thought leaders in tower and infrastructure companies</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Best thought leaders in streaming and digital media</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Best thought leaders in advertising and creative agencies</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Best thought leaders in pr firms</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Best thought leaders in retail and consumer goods</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Best thought leaders in large retail chains</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Best thought leaders in fmcg companies</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Best thought leaders in e-commerce platforms</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Best thought leaders in transport and logistics</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Best thought leaders in airlines</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Best thought leaders in freight and logistics</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Best thought leaders in ports and shipping</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Best thought leaders in agriculture and agribusiness</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Best thought leaders in large-scale farming operations</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Best thought leaders in agricultural cooperatives</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Best thought leaders in food processing</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Best thought leaders in hotel chains</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Best thought leaders in casino and gaming</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Best thought leaders in event management companies</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Best chief executive officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Best chief people officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Best chief human resources officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Best chief learning officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Best chief operating officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Best chief financial officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Best chief of staffs to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Best chief development officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Best managing partners to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Best senior partners to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Best practice group leaders to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Best operating partners (pe) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Best human capital partners (pe) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Best portfolio talent partners (pe) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Best vp of peoples to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Best vp of talent developments to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Best vp of organizational developments to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Best head of learning and developments to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Best head of talent managements to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Best head of leadership developments to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Best director of people and cultures to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Best director of operationses to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Best regional managing directors to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Best division heads to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Best business unit leaders to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Best general managers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Best country managers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Best managing directors to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Best board chairs to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Best deputy board chairs to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Best executive directors (nonprofit) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Best principals (schools) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Best head of schools to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Best deans (university) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Best provosts to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Best conference directors to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Best event directors to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Best executive assistant to ceos to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Best founders to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Best co-founders to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Best presidents to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Best senior vice presidents to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Best partners (law) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Best partners (accounting) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Best partners (consulting) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Best school association executive directors to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Best superintendents (school districts) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Best chief medical officers (healthcare) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Best chief nursing officers (healthcare) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Best vp of medical affairses to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Best hospital administrators to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Best chief strategy officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Best chief transformation officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Best head of change managements to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Best head of diversity and inclusions to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Best family office principals to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Best family office chief investment officers to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Best trustees to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Best program directors (nonprofit) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Best head of capacity buildings (nonprofit) to follow for thought leadership</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>COMMERCIAL</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in supply chain -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2186,7 +2186,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in supply chain -> PUBLISHED + LinkedIn post + handoff
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2186,13 +2186,36 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>PUBLISHED</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-best-thought-leaders-in-supply-chain-20260327</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>5990</v>
       </c>
     </row>
     <row r="45">

</xml_diff>

<commit_message>
Update blog queue: Best thought leaders in logistics -> WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2231,7 +2231,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update blog queue: logistics->SKIP, procurement->WRITING
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2231,12 +2231,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Already exists: consultclarity.org/post/thought-leaders-logistics-leadership</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2258,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>WRITING</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add blog content and update queue: procurement -> WRITTEN
</commit_message>
<xml_diff>
--- a/blog-data/blog-queue.xlsx
+++ b/blog-data/blog-queue.xlsx
@@ -2258,13 +2258,31 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>WRITING</t>
+          <t>WRITTEN</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ADJACENT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://github.com/jonno-alt/social-images/tree/main/blog-images/blog-procurement-20260327</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>5250</v>
       </c>
     </row>
     <row r="47">

</xml_diff>